<commit_message>
updated logic for writing to excel3 sheet for excelwrite1 and excelwrite2
</commit_message>
<xml_diff>
--- a/SeleniumFramework9/Excels/DataSheet2.xlsx
+++ b/SeleniumFramework9/Excels/DataSheet2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\git\DemoWebShop1\SeleniumFramework9\Excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Selenium\DemoWebShop1\DemoWebShop1\SeleniumFramework9\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45F8871A-8C34-419B-BF14-348932D06FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891F8D21-FF49-47AF-9FAD-F1AE73678BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>FirstName</t>
   </si>
@@ -46,49 +46,40 @@
     <t>Login Status</t>
   </si>
   <si>
-    <t>acg854</t>
-  </si>
-  <si>
     <t>def</t>
   </si>
   <si>
-    <t>acg854@gmail.com</t>
-  </si>
-  <si>
     <t>Password123</t>
   </si>
   <si>
     <t>Male</t>
   </si>
   <si>
-    <t>ghi135</t>
-  </si>
-  <si>
     <t>jkl</t>
   </si>
   <si>
-    <t>ghi135135@gmail.com</t>
-  </si>
-  <si>
     <t>Female</t>
   </si>
   <si>
-    <t>mno135</t>
-  </si>
-  <si>
-    <t>pqr</t>
-  </si>
-  <si>
-    <t>mno135135@gmail.com</t>
-  </si>
-  <si>
-    <t>stu135</t>
-  </si>
-  <si>
     <t>vwx</t>
   </si>
   <si>
-    <t>stu135135@gmail.com</t>
+    <t>stun13512@gmail.com</t>
+  </si>
+  <si>
+    <t>acdg854</t>
+  </si>
+  <si>
+    <t>acdg854@gmail.com</t>
+  </si>
+  <si>
+    <t>jhm1362</t>
+  </si>
+  <si>
+    <t>jhm1252@gmail.com</t>
+  </si>
+  <si>
+    <t>stun2512</t>
   </si>
 </sst>
 </file>
@@ -451,8 +442,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="7" max="7" width="28.77734375" customWidth="1"/>
+    <col min="8" max="8" width="19.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -482,90 +481,69 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{634668E1-17BC-468C-BAA3-44FEDDF18BE6}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{92F568B4-2959-4125-9030-70B451A52CCB}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{84C841B0-8B71-460D-AFC0-6262DB07F5B9}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{AC779810-A7B1-40AC-AF47-EC3334C6C12B}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{0D842573-D354-4201-9460-627149A13940}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{8D24FA9C-E2A8-428F-98A8-E71403B1F8A2}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{4D900A81-6316-4106-A293-AC10B4C44AA6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
New Code Added UserTest2
</commit_message>
<xml_diff>
--- a/SeleniumFramework9/Excels/DataSheet2.xlsx
+++ b/SeleniumFramework9/Excels/DataSheet2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Selenium\DemoWebShop1\DemoWebShop1\SeleniumFramework9\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891F8D21-FF49-47AF-9FAD-F1AE73678BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCA46A7-28A7-4965-B846-6DACC8FE54AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>FirstName</t>
   </si>
@@ -46,40 +46,49 @@
     <t>Login Status</t>
   </si>
   <si>
+    <t>acg854</t>
+  </si>
+  <si>
     <t>def</t>
   </si>
   <si>
+    <t>acg854@gmail.com</t>
+  </si>
+  <si>
     <t>Password123</t>
   </si>
   <si>
     <t>Male</t>
   </si>
   <si>
+    <t>ghi135</t>
+  </si>
+  <si>
     <t>jkl</t>
   </si>
   <si>
+    <t>ghi135135@gmail.com</t>
+  </si>
+  <si>
     <t>Female</t>
   </si>
   <si>
+    <t>mno135</t>
+  </si>
+  <si>
+    <t>pqr</t>
+  </si>
+  <si>
+    <t>mno135135@gmail.com</t>
+  </si>
+  <si>
+    <t>stu135</t>
+  </si>
+  <si>
     <t>vwx</t>
   </si>
   <si>
-    <t>stun13512@gmail.com</t>
-  </si>
-  <si>
-    <t>acdg854</t>
-  </si>
-  <si>
-    <t>acdg854@gmail.com</t>
-  </si>
-  <si>
-    <t>jhm1362</t>
-  </si>
-  <si>
-    <t>jhm1252@gmail.com</t>
-  </si>
-  <si>
-    <t>stun2512</t>
+    <t>stu135135@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -442,15 +451,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
-    <col min="7" max="7" width="28.77734375" customWidth="1"/>
-    <col min="8" max="8" width="19.21875" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -481,69 +489,90 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{0D842573-D354-4201-9460-627149A13940}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{8D24FA9C-E2A8-428F-98A8-E71403B1F8A2}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{4D900A81-6316-4106-A293-AC10B4C44AA6}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{9B8F145B-52C5-4815-B07C-995F2DF18E4D}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{19DFC721-353A-4F93-A05A-2065F2F6DD95}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{2BFF0941-0F6B-4A16-915A-6A7D6747E5BB}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{40B21063-5F1E-4AAF-B716-4B51BE783DDF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>